<commit_message>
Back-translation, second run: move judgements and notes one column right (entered in flag_qwen and judgement by mistake; values unchanged); add the judging rules, given to the author before judging
</commit_message>
<xml_diff>
--- a/data/translation/equivalence_judgement_20260929_0650.xlsx
+++ b/data/translation/equivalence_judgement_20260929_0650.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1580" uniqueCount="530">
   <si>
     <t>item_id</t>
   </si>
@@ -1635,7 +1635,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1654,13 +1654,6 @@
       <sz val="10"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -2125,28 +2118,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2155,118 +2151,115 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2731,13 +2724,11 @@
       <c r="M2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="3"/>
+      <c r="O2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2781,13 +2772,11 @@
       <c r="M3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2831,13 +2820,11 @@
       <c r="M4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P4" s="2" t="s">
+      <c r="P4" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2881,13 +2868,11 @@
       <c r="M5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P5" s="2" t="s">
+      <c r="P5" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2931,13 +2916,11 @@
       <c r="M6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="3"/>
+      <c r="O6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P6" s="2" t="s">
+      <c r="P6" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2981,13 +2964,11 @@
       <c r="M7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="N7" s="3"/>
+      <c r="O7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P7" s="2" t="s">
+      <c r="P7" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3031,13 +3012,11 @@
       <c r="M8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="3"/>
+      <c r="O8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P8" s="2" t="s">
+      <c r="P8" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3081,13 +3060,11 @@
       <c r="M9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="N9" s="3"/>
+      <c r="O9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P9" s="2" t="s">
+      <c r="P9" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3131,13 +3108,11 @@
       <c r="M10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="3"/>
+      <c r="O10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3181,13 +3156,11 @@
       <c r="M11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N11" s="3" t="s">
+      <c r="N11" s="3"/>
+      <c r="O11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3231,13 +3204,11 @@
       <c r="M12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N12" s="3" t="s">
+      <c r="N12" s="3"/>
+      <c r="O12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P12" s="2" t="s">
+      <c r="P12" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3281,13 +3252,11 @@
       <c r="M13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N13" s="3" t="s">
+      <c r="N13" s="3"/>
+      <c r="O13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P13" s="2" t="s">
+      <c r="P13" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3331,13 +3300,11 @@
       <c r="M14" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N14" s="3" t="s">
+      <c r="N14" s="3"/>
+      <c r="O14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P14" s="2" t="s">
+      <c r="P14" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3381,13 +3348,11 @@
       <c r="M15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="N15" s="3"/>
+      <c r="O15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P15" s="2" t="s">
+      <c r="P15" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3431,13 +3396,11 @@
       <c r="M16" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="N16" s="3"/>
+      <c r="O16" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O16" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3481,13 +3444,11 @@
       <c r="M17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="N17" s="3"/>
+      <c r="O17" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3531,13 +3492,11 @@
       <c r="M18" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="N18" s="3"/>
+      <c r="O18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P18" s="2" t="s">
+      <c r="P18" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3581,13 +3540,11 @@
       <c r="M19" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N19" s="3" t="s">
+      <c r="N19" s="3"/>
+      <c r="O19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O19" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P19" s="2" t="s">
+      <c r="P19" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3631,13 +3588,11 @@
       <c r="M20" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N20" s="3" t="s">
+      <c r="N20" s="3"/>
+      <c r="O20" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P20" s="2" t="s">
+      <c r="P20" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3681,13 +3636,11 @@
       <c r="M21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N21" s="3" t="s">
+      <c r="N21" s="3"/>
+      <c r="O21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O21" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P21" s="2" t="s">
+      <c r="P21" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3731,13 +3684,11 @@
       <c r="M22" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N22" s="3" t="s">
+      <c r="N22" s="3"/>
+      <c r="O22" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P22" s="2" t="s">
+      <c r="P22" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3781,13 +3732,11 @@
       <c r="M23" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N23" s="3" t="s">
+      <c r="N23" s="3"/>
+      <c r="O23" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O23" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P23" s="2" t="s">
+      <c r="P23" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3831,13 +3780,11 @@
       <c r="M24" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="3" t="s">
+      <c r="N24" s="3"/>
+      <c r="O24" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P24" s="2" t="s">
+      <c r="P24" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3881,13 +3828,11 @@
       <c r="M25" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N25" s="3" t="s">
+      <c r="N25" s="3"/>
+      <c r="O25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O25" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="P25" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3931,13 +3876,11 @@
       <c r="M26" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N26" s="3" t="s">
+      <c r="N26" s="3"/>
+      <c r="O26" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="P26" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3981,13 +3924,11 @@
       <c r="M27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N27" s="3" t="s">
+      <c r="N27" s="3"/>
+      <c r="O27" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O27" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="P27" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4031,13 +3972,11 @@
       <c r="M28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N28" s="3" t="s">
+      <c r="N28" s="3"/>
+      <c r="O28" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O28" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="P28" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4081,13 +4020,11 @@
       <c r="M29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N29" s="3" t="s">
+      <c r="N29" s="3"/>
+      <c r="O29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O29" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="P29" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4131,13 +4068,11 @@
       <c r="M30" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N30" s="3" t="s">
+      <c r="N30" s="3"/>
+      <c r="O30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O30" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="P30" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4181,13 +4116,11 @@
       <c r="M31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N31" s="3" t="s">
+      <c r="N31" s="3"/>
+      <c r="O31" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O31" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="P31" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4231,13 +4164,11 @@
       <c r="M32" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N32" s="3" t="s">
+      <c r="N32" s="3"/>
+      <c r="O32" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O32" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="P32" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4281,13 +4212,11 @@
       <c r="M33" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N33" s="3" t="s">
+      <c r="N33" s="3"/>
+      <c r="O33" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O33" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="P33" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4331,13 +4260,11 @@
       <c r="M34" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N34" s="3" t="s">
+      <c r="N34" s="3"/>
+      <c r="O34" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O34" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="P34" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4381,13 +4308,11 @@
       <c r="M35" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N35" s="3" t="s">
+      <c r="N35" s="3"/>
+      <c r="O35" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O35" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P35" s="2" t="s">
+      <c r="P35" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4431,13 +4356,11 @@
       <c r="M36" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N36" s="3" t="s">
+      <c r="N36" s="3"/>
+      <c r="O36" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O36" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P36" s="2" t="s">
+      <c r="P36" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4481,13 +4404,11 @@
       <c r="M37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N37" s="3" t="s">
+      <c r="N37" s="3"/>
+      <c r="O37" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O37" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P37" s="2" t="s">
+      <c r="P37" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -4531,14 +4452,12 @@
       <c r="M38" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N38" s="3" t="s">
+      <c r="N38" s="3"/>
+      <c r="O38" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O38" s="4" t="s">
+      <c r="P38" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P38" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="39" ht="315" spans="1:16">
@@ -4581,14 +4500,12 @@
       <c r="M39" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N39" s="3" t="s">
+      <c r="N39" s="3"/>
+      <c r="O39" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O39" s="4" t="s">
+      <c r="P39" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P39" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="40" ht="315" spans="1:16">
@@ -4631,14 +4548,12 @@
       <c r="M40" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N40" s="3" t="s">
+      <c r="N40" s="3"/>
+      <c r="O40" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O40" s="4" t="s">
+      <c r="P40" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P40" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="41" ht="315" spans="1:16">
@@ -4681,14 +4596,12 @@
       <c r="M41" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N41" s="3" t="s">
+      <c r="N41" s="3"/>
+      <c r="O41" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O41" s="4" t="s">
+      <c r="P41" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P41" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="42" ht="315" spans="1:16">
@@ -4731,14 +4644,12 @@
       <c r="M42" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N42" s="3" t="s">
+      <c r="N42" s="3"/>
+      <c r="O42" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O42" s="4" t="s">
+      <c r="P42" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P42" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="43" ht="315" spans="1:16">
@@ -4781,14 +4692,12 @@
       <c r="M43" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N43" s="3" t="s">
+      <c r="N43" s="3"/>
+      <c r="O43" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O43" s="4" t="s">
+      <c r="P43" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P43" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="44" ht="315" spans="1:16">
@@ -4831,14 +4740,12 @@
       <c r="M44" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N44" s="3" t="s">
+      <c r="N44" s="3"/>
+      <c r="O44" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O44" s="4" t="s">
+      <c r="P44" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P44" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="45" ht="315" spans="1:16">
@@ -4881,14 +4788,12 @@
       <c r="M45" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N45" s="3" t="s">
+      <c r="N45" s="3"/>
+      <c r="O45" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O45" s="4" t="s">
+      <c r="P45" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P45" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="46" ht="315" spans="1:16">
@@ -4931,14 +4836,12 @@
       <c r="M46" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N46" s="3" t="s">
+      <c r="N46" s="3"/>
+      <c r="O46" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O46" s="4" t="s">
+      <c r="P46" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="P46" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="47" ht="300" spans="1:16">
@@ -4981,14 +4884,12 @@
       <c r="M47" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N47" s="3" t="s">
+      <c r="N47" s="3"/>
+      <c r="O47" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O47" s="4" t="s">
+      <c r="P47" s="4" t="s">
         <v>240</v>
-      </c>
-      <c r="P47" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="48" ht="28.8" spans="1:16">
@@ -5031,13 +4932,11 @@
       <c r="M48" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N48" s="3" t="s">
+      <c r="N48" s="3"/>
+      <c r="O48" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O48" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P48" s="2" t="s">
+      <c r="P48" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5081,13 +4980,11 @@
       <c r="M49" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N49" s="3" t="s">
+      <c r="N49" s="3"/>
+      <c r="O49" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O49" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P49" s="2" t="s">
+      <c r="P49" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5131,14 +5028,12 @@
       <c r="M50" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N50" s="3" t="s">
+      <c r="N50" s="3"/>
+      <c r="O50" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O50" s="4" t="s">
+      <c r="P50" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P50" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="51" ht="372" spans="1:16">
@@ -5181,14 +5076,12 @@
       <c r="M51" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N51" s="3" t="s">
+      <c r="N51" s="3"/>
+      <c r="O51" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O51" s="4" t="s">
+      <c r="P51" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P51" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="52" ht="372" spans="1:16">
@@ -5231,14 +5124,12 @@
       <c r="M52" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N52" s="3" t="s">
+      <c r="N52" s="3"/>
+      <c r="O52" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O52" s="4" t="s">
+      <c r="P52" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P52" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="53" ht="372" spans="1:16">
@@ -5281,14 +5172,12 @@
       <c r="M53" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N53" s="3" t="s">
+      <c r="N53" s="3"/>
+      <c r="O53" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O53" s="4" t="s">
+      <c r="P53" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P53" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="54" ht="372" spans="1:16">
@@ -5331,14 +5220,12 @@
       <c r="M54" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N54" s="3" t="s">
+      <c r="N54" s="3"/>
+      <c r="O54" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O54" s="4" t="s">
+      <c r="P54" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P54" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="55" ht="372" spans="1:16">
@@ -5381,14 +5268,12 @@
       <c r="M55" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N55" s="3" t="s">
+      <c r="N55" s="3"/>
+      <c r="O55" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O55" s="4" t="s">
+      <c r="P55" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P55" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="56" ht="372" spans="1:16">
@@ -5431,14 +5316,12 @@
       <c r="M56" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N56" s="3" t="s">
+      <c r="N56" s="3"/>
+      <c r="O56" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O56" s="4" t="s">
+      <c r="P56" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P56" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="57" ht="372" spans="1:16">
@@ -5481,14 +5364,12 @@
       <c r="M57" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N57" s="3" t="s">
+      <c r="N57" s="3"/>
+      <c r="O57" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O57" s="4" t="s">
+      <c r="P57" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P57" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="58" ht="372" spans="1:16">
@@ -5531,14 +5412,12 @@
       <c r="M58" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N58" s="3" t="s">
+      <c r="N58" s="3"/>
+      <c r="O58" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O58" s="4" t="s">
+      <c r="P58" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="P58" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="59" ht="372" spans="1:16">
@@ -5581,14 +5460,12 @@
       <c r="M59" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N59" s="3" t="s">
+      <c r="N59" s="3"/>
+      <c r="O59" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O59" s="4" t="s">
+      <c r="P59" s="4" t="s">
         <v>296</v>
-      </c>
-      <c r="P59" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="60" ht="357" spans="1:16">
@@ -5631,14 +5508,12 @@
       <c r="M60" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N60" s="3" t="s">
+      <c r="N60" s="3"/>
+      <c r="O60" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O60" s="4" t="s">
+      <c r="P60" s="4" t="s">
         <v>302</v>
-      </c>
-      <c r="P60" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="61" ht="357" spans="1:16">
@@ -5681,14 +5556,12 @@
       <c r="M61" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N61" s="3" t="s">
+      <c r="N61" s="3"/>
+      <c r="O61" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O61" s="4" t="s">
+      <c r="P61" s="4" t="s">
         <v>305</v>
-      </c>
-      <c r="P61" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="62" ht="57.6" spans="1:16">
@@ -5731,13 +5604,11 @@
       <c r="M62" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N62" s="3" t="s">
+      <c r="N62" s="3"/>
+      <c r="O62" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O62" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P62" s="2" t="s">
+      <c r="P62" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5781,13 +5652,11 @@
       <c r="M63" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N63" s="3" t="s">
+      <c r="N63" s="3"/>
+      <c r="O63" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O63" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P63" s="2" t="s">
+      <c r="P63" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5831,13 +5700,11 @@
       <c r="M64" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N64" s="3" t="s">
+      <c r="N64" s="3"/>
+      <c r="O64" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O64" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P64" s="2" t="s">
+      <c r="P64" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5881,13 +5748,11 @@
       <c r="M65" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N65" s="3" t="s">
+      <c r="N65" s="3"/>
+      <c r="O65" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O65" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P65" s="2" t="s">
+      <c r="P65" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5931,13 +5796,11 @@
       <c r="M66" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N66" s="3" t="s">
+      <c r="N66" s="3"/>
+      <c r="O66" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O66" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P66" s="2" t="s">
+      <c r="P66" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5981,13 +5844,11 @@
       <c r="M67" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N67" s="3" t="s">
+      <c r="N67" s="3"/>
+      <c r="O67" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O67" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P67" s="2" t="s">
+      <c r="P67" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6031,13 +5892,11 @@
       <c r="M68" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N68" s="3" t="s">
+      <c r="N68" s="3"/>
+      <c r="O68" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O68" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P68" s="2" t="s">
+      <c r="P68" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6081,13 +5940,11 @@
       <c r="M69" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N69" s="3" t="s">
+      <c r="N69" s="3"/>
+      <c r="O69" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O69" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P69" s="2" t="s">
+      <c r="P69" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6131,13 +5988,11 @@
       <c r="M70" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N70" s="3" t="s">
+      <c r="N70" s="3"/>
+      <c r="O70" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O70" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P70" s="2" t="s">
+      <c r="P70" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6181,13 +6036,11 @@
       <c r="M71" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N71" s="3" t="s">
+      <c r="N71" s="3"/>
+      <c r="O71" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O71" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P71" s="2" t="s">
+      <c r="P71" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6231,14 +6084,12 @@
       <c r="M72" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N72" s="3" t="s">
+      <c r="N72" s="3"/>
+      <c r="O72" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O72" s="4" t="s">
+      <c r="P72" s="4" t="s">
         <v>359</v>
-      </c>
-      <c r="P72" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="73" ht="297" spans="1:16">
@@ -6281,14 +6132,12 @@
       <c r="M73" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N73" s="3" t="s">
+      <c r="N73" s="3"/>
+      <c r="O73" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O73" s="4" t="s">
+      <c r="P73" s="4" t="s">
         <v>363</v>
-      </c>
-      <c r="P73" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="74" ht="57.6" spans="1:16">
@@ -6331,13 +6180,11 @@
       <c r="M74" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N74" s="3" t="s">
+      <c r="N74" s="3"/>
+      <c r="O74" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O74" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P74" s="2" t="s">
+      <c r="P74" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6381,13 +6228,11 @@
       <c r="M75" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N75" s="3" t="s">
+      <c r="N75" s="3"/>
+      <c r="O75" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O75" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P75" s="2" t="s">
+      <c r="P75" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6431,13 +6276,11 @@
       <c r="M76" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N76" s="3" t="s">
+      <c r="N76" s="3"/>
+      <c r="O76" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O76" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P76" s="2" t="s">
+      <c r="P76" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6481,13 +6324,11 @@
       <c r="M77" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N77" s="3" t="s">
+      <c r="N77" s="3"/>
+      <c r="O77" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O77" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P77" s="2" t="s">
+      <c r="P77" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6531,13 +6372,11 @@
       <c r="M78" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N78" s="3" t="s">
+      <c r="N78" s="3"/>
+      <c r="O78" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O78" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P78" s="2" t="s">
+      <c r="P78" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6581,13 +6420,11 @@
       <c r="M79" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N79" s="3" t="s">
+      <c r="N79" s="3"/>
+      <c r="O79" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O79" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P79" s="2" t="s">
+      <c r="P79" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6631,13 +6468,11 @@
       <c r="M80" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N80" s="3" t="s">
+      <c r="N80" s="3"/>
+      <c r="O80" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O80" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P80" s="2" t="s">
+      <c r="P80" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6681,13 +6516,11 @@
       <c r="M81" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N81" s="3" t="s">
+      <c r="N81" s="3"/>
+      <c r="O81" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O81" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P81" s="2" t="s">
+      <c r="P81" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6731,13 +6564,11 @@
       <c r="M82" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N82" s="3" t="s">
+      <c r="N82" s="3"/>
+      <c r="O82" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O82" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P82" s="2" t="s">
+      <c r="P82" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6781,13 +6612,11 @@
       <c r="M83" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N83" s="3" t="s">
+      <c r="N83" s="3"/>
+      <c r="O83" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O83" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P83" s="2" t="s">
+      <c r="P83" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6831,14 +6660,12 @@
       <c r="M84" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N84" s="3" t="s">
+      <c r="N84" s="3"/>
+      <c r="O84" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O84" s="4" t="s">
+      <c r="P84" s="4" t="s">
         <v>415</v>
-      </c>
-      <c r="P84" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="85" ht="282" spans="1:16">
@@ -6881,14 +6708,12 @@
       <c r="M85" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N85" s="3" t="s">
+      <c r="N85" s="3"/>
+      <c r="O85" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O85" s="4" t="s">
+      <c r="P85" s="4" t="s">
         <v>419</v>
-      </c>
-      <c r="P85" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="86" ht="57.6" spans="1:16">
@@ -6931,13 +6756,11 @@
       <c r="M86" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N86" s="3" t="s">
+      <c r="N86" s="3"/>
+      <c r="O86" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O86" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P86" s="2" t="s">
+      <c r="P86" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6981,13 +6804,11 @@
       <c r="M87" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N87" s="3" t="s">
+      <c r="N87" s="3"/>
+      <c r="O87" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O87" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P87" s="2" t="s">
+      <c r="P87" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7031,13 +6852,11 @@
       <c r="M88" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N88" s="3" t="s">
+      <c r="N88" s="3"/>
+      <c r="O88" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O88" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P88" s="2" t="s">
+      <c r="P88" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7081,13 +6900,11 @@
       <c r="M89" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N89" s="3" t="s">
+      <c r="N89" s="3"/>
+      <c r="O89" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O89" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P89" s="2" t="s">
+      <c r="P89" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7131,13 +6948,11 @@
       <c r="M90" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N90" s="3" t="s">
+      <c r="N90" s="3"/>
+      <c r="O90" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O90" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P90" s="2" t="s">
+      <c r="P90" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7181,13 +6996,11 @@
       <c r="M91" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N91" s="3" t="s">
+      <c r="N91" s="3"/>
+      <c r="O91" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O91" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P91" s="2" t="s">
+      <c r="P91" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7231,13 +7044,11 @@
       <c r="M92" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N92" s="3" t="s">
+      <c r="N92" s="3"/>
+      <c r="O92" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O92" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P92" s="2" t="s">
+      <c r="P92" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7281,13 +7092,11 @@
       <c r="M93" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N93" s="3" t="s">
+      <c r="N93" s="3"/>
+      <c r="O93" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O93" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P93" s="2" t="s">
+      <c r="P93" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7331,13 +7140,11 @@
       <c r="M94" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N94" s="3" t="s">
+      <c r="N94" s="3"/>
+      <c r="O94" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O94" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P94" s="2" t="s">
+      <c r="P94" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7381,13 +7188,11 @@
       <c r="M95" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N95" s="3" t="s">
+      <c r="N95" s="3"/>
+      <c r="O95" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O95" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P95" s="2" t="s">
+      <c r="P95" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7431,13 +7236,11 @@
       <c r="M96" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N96" s="3" t="s">
+      <c r="N96" s="3"/>
+      <c r="O96" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O96" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P96" s="2" t="s">
+      <c r="P96" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7481,13 +7284,11 @@
       <c r="M97" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N97" s="3" t="s">
+      <c r="N97" s="3"/>
+      <c r="O97" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O97" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P97" s="2" t="s">
+      <c r="P97" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7531,13 +7332,11 @@
       <c r="M98" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N98" s="3" t="s">
+      <c r="N98" s="3"/>
+      <c r="O98" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O98" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P98" s="2" t="s">
+      <c r="P98" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7581,13 +7380,11 @@
       <c r="M99" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N99" s="3" t="s">
+      <c r="N99" s="3"/>
+      <c r="O99" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O99" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P99" s="2" t="s">
+      <c r="P99" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7631,13 +7428,11 @@
       <c r="M100" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N100" s="3" t="s">
+      <c r="N100" s="3"/>
+      <c r="O100" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O100" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P100" s="2" t="s">
+      <c r="P100" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7681,13 +7476,11 @@
       <c r="M101" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N101" s="3" t="s">
+      <c r="N101" s="3"/>
+      <c r="O101" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O101" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P101" s="2" t="s">
+      <c r="P101" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7731,13 +7524,11 @@
       <c r="M102" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N102" s="3" t="s">
+      <c r="N102" s="3"/>
+      <c r="O102" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O102" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P102" s="2" t="s">
+      <c r="P102" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7781,13 +7572,11 @@
       <c r="M103" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N103" s="3" t="s">
+      <c r="N103" s="3"/>
+      <c r="O103" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O103" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P103" s="2" t="s">
+      <c r="P103" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7831,13 +7620,11 @@
       <c r="M104" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N104" s="3" t="s">
+      <c r="N104" s="3"/>
+      <c r="O104" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O104" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P104" s="2" t="s">
+      <c r="P104" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7881,13 +7668,11 @@
       <c r="M105" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N105" s="3" t="s">
+      <c r="N105" s="3"/>
+      <c r="O105" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O105" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P105" s="2" t="s">
+      <c r="P105" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -7931,14 +7716,12 @@
       <c r="M106" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N106" s="3" t="s">
+      <c r="N106" s="3"/>
+      <c r="O106" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O106" s="4" t="s">
+      <c r="P106" s="4" t="s">
         <v>508</v>
-      </c>
-      <c r="P106" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="107" ht="315" spans="1:16">
@@ -7981,14 +7764,12 @@
       <c r="M107" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N107" s="3" t="s">
+      <c r="N107" s="3"/>
+      <c r="O107" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="O107" s="4" t="s">
+      <c r="P107" s="4" t="s">
         <v>511</v>
-      </c>
-      <c r="P107" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="108" ht="28.8" spans="1:16">
@@ -8031,13 +7812,11 @@
       <c r="M108" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N108" s="3" t="s">
+      <c r="N108" s="3"/>
+      <c r="O108" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O108" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P108" s="2" t="s">
+      <c r="P108" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -8081,13 +7860,11 @@
       <c r="M109" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="N109" s="3" t="s">
+      <c r="N109" s="3"/>
+      <c r="O109" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O109" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="P109" s="2" t="s">
+      <c r="P109" s="4" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>